<commit_message>
Modify the damping matrices assembly
</commit_message>
<xml_diff>
--- a/validation/data/particle_velocity/results/silencer/WB_results_silencer_DB_Vn1_Z1_Z2_20mm.xlsx
+++ b/validation/data/particle_velocity/results/silencer/WB_results_silencer_DB_Vn1_Z1_Z2_20mm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorios\VIBRA\validation\data\particle_velocity\results\silencer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62278094-FD26-405F-8F67-9187AD0B7955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E5F7B8-AF0A-4EF0-84D2-496FE1BFE3C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="5" xr2:uid="{663DECE1-D11E-44CD-A079-C79636EAEC85}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11385" xr2:uid="{663DECE1-D11E-44CD-A079-C79636EAEC85}"/>
   </bookViews>
   <sheets>
     <sheet name="input_face_pressure" sheetId="1" r:id="rId1"/>
@@ -12877,7 +12877,7 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>0.58145000000000002</v>
+        <v>0.56859999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -12885,7 +12885,7 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>1.6904999999999999</v>
+        <v>1.6667000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -12893,7 +12893,7 @@
         <v>15</v>
       </c>
       <c r="B4">
-        <v>2.3713000000000002</v>
+        <v>2.3443000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -12901,7 +12901,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>2.5171999999999999</v>
+        <v>2.4942000000000002</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -12909,7 +12909,7 @@
         <v>25</v>
       </c>
       <c r="B6">
-        <v>2.6741000000000001</v>
+        <v>2.6570999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -12917,7 +12917,7 @@
         <v>30</v>
       </c>
       <c r="B7">
-        <v>3.4085999999999999</v>
+        <v>3.3919000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -12925,7 +12925,7 @@
         <v>35</v>
       </c>
       <c r="B8">
-        <v>4.5838000000000001</v>
+        <v>4.5613999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -12933,7 +12933,7 @@
         <v>40</v>
       </c>
       <c r="B9">
-        <v>5.6957000000000004</v>
+        <v>5.6668000000000003</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -12941,7 +12941,7 @@
         <v>45</v>
       </c>
       <c r="B10">
-        <v>6.5003000000000002</v>
+        <v>6.4669999999999996</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -12949,7 +12949,7 @@
         <v>50</v>
       </c>
       <c r="B11">
-        <v>7.0561999999999996</v>
+        <v>7.0235000000000003</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -12957,7 +12957,7 @@
         <v>55</v>
       </c>
       <c r="B12">
-        <v>7.5938999999999997</v>
+        <v>7.5696000000000003</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -12965,7 +12965,7 @@
         <v>60</v>
       </c>
       <c r="B13">
-        <v>8.3446999999999996</v>
+        <v>8.3366000000000007</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -12973,7 +12973,7 @@
         <v>65</v>
       </c>
       <c r="B14">
-        <v>9.3527000000000005</v>
+        <v>9.3629999999999995</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -12981,7 +12981,7 @@
         <v>70</v>
       </c>
       <c r="B15">
-        <v>10.468</v>
+        <v>10.494</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -12989,7 +12989,7 @@
         <v>75</v>
       </c>
       <c r="B16">
-        <v>11.519</v>
+        <v>11.555</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -12997,7 +12997,7 @@
         <v>80</v>
       </c>
       <c r="B17">
-        <v>12.416</v>
+        <v>12.462</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -13005,7 +13005,7 @@
         <v>85</v>
       </c>
       <c r="B18">
-        <v>13.164999999999999</v>
+        <v>13.221</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -13013,7 +13013,7 @@
         <v>90</v>
       </c>
       <c r="B19">
-        <v>13.824999999999999</v>
+        <v>13.894</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -13021,7 +13021,7 @@
         <v>95</v>
       </c>
       <c r="B20">
-        <v>14.471</v>
+        <v>14.555999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -13029,7 +13029,7 @@
         <v>100</v>
       </c>
       <c r="B21">
-        <v>15.156000000000001</v>
+        <v>15.259</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -13037,7 +13037,7 @@
         <v>105</v>
       </c>
       <c r="B22">
-        <v>15.884</v>
+        <v>16.004000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -13045,7 +13045,7 @@
         <v>110</v>
       </c>
       <c r="B23">
-        <v>16.62</v>
+        <v>16.754000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -13053,7 +13053,7 @@
         <v>115</v>
       </c>
       <c r="B24">
-        <v>17.312999999999999</v>
+        <v>17.456</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -13061,7 +13061,7 @@
         <v>120</v>
       </c>
       <c r="B25">
-        <v>17.922999999999998</v>
+        <v>18.071999999999999</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -13069,7 +13069,7 @@
         <v>125</v>
       </c>
       <c r="B26">
-        <v>18.433</v>
+        <v>18.585999999999999</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -13077,7 +13077,7 @@
         <v>130</v>
       </c>
       <c r="B27">
-        <v>18.844999999999999</v>
+        <v>19.001000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -13085,7 +13085,7 @@
         <v>135</v>
       </c>
       <c r="B28">
-        <v>19.178000000000001</v>
+        <v>19.338000000000001</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -13093,7 +13093,7 @@
         <v>140</v>
       </c>
       <c r="B29">
-        <v>19.459</v>
+        <v>19.623000000000001</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -13101,7 +13101,7 @@
         <v>145</v>
       </c>
       <c r="B30">
-        <v>19.716000000000001</v>
+        <v>19.885000000000002</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -13109,7 +13109,7 @@
         <v>150</v>
       </c>
       <c r="B31">
-        <v>19.971</v>
+        <v>20.143999999999998</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -13117,7 +13117,7 @@
         <v>155</v>
       </c>
       <c r="B32">
-        <v>20.236000000000001</v>
+        <v>20.414999999999999</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -13125,7 +13125,7 @@
         <v>160</v>
       </c>
       <c r="B33">
-        <v>20.518000000000001</v>
+        <v>20.702999999999999</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -13133,7 +13133,7 @@
         <v>165</v>
       </c>
       <c r="B34">
-        <v>20.815999999999999</v>
+        <v>21.01</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -13141,7 +13141,7 @@
         <v>170</v>
       </c>
       <c r="B35">
-        <v>21.132000000000001</v>
+        <v>21.335999999999999</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -13149,7 +13149,7 @@
         <v>175</v>
       </c>
       <c r="B36">
-        <v>21.466999999999999</v>
+        <v>21.683</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -13157,7 +13157,7 @@
         <v>180</v>
       </c>
       <c r="B37">
-        <v>21.824000000000002</v>
+        <v>22.053999999999998</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -13165,7 +13165,7 @@
         <v>185</v>
       </c>
       <c r="B38">
-        <v>22.206</v>
+        <v>22.454000000000001</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -13173,7 +13173,7 @@
         <v>190</v>
       </c>
       <c r="B39">
-        <v>22.614000000000001</v>
+        <v>22.882000000000001</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -13181,7 +13181,7 @@
         <v>195</v>
       </c>
       <c r="B40">
-        <v>23.047000000000001</v>
+        <v>23.335999999999999</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -13189,7 +13189,7 @@
         <v>200</v>
       </c>
       <c r="B41">
-        <v>23.501000000000001</v>
+        <v>23.812000000000001</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -13197,7 +13197,7 @@
         <v>205</v>
       </c>
       <c r="B42">
-        <v>23.97</v>
+        <v>24.303000000000001</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -13205,7 +13205,7 @@
         <v>210</v>
       </c>
       <c r="B43">
-        <v>24.448</v>
+        <v>24.803000000000001</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -13213,7 +13213,7 @@
         <v>215</v>
       </c>
       <c r="B44">
-        <v>24.928000000000001</v>
+        <v>25.305</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -13221,7 +13221,7 @@
         <v>220</v>
       </c>
       <c r="B45">
-        <v>25.405000000000001</v>
+        <v>25.802</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -13229,7 +13229,7 @@
         <v>225</v>
       </c>
       <c r="B46">
-        <v>25.875</v>
+        <v>26.291</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -13237,7 +13237,7 @@
         <v>230</v>
       </c>
       <c r="B47">
-        <v>26.334</v>
+        <v>26.768999999999998</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -13245,7 +13245,7 @@
         <v>235</v>
       </c>
       <c r="B48">
-        <v>26.780999999999999</v>
+        <v>27.233000000000001</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -13253,7 +13253,7 @@
         <v>240</v>
       </c>
       <c r="B49">
-        <v>27.215</v>
+        <v>27.684000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -13261,7 +13261,7 @@
         <v>245</v>
       </c>
       <c r="B50">
-        <v>27.638000000000002</v>
+        <v>28.122</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -13269,7 +13269,7 @@
         <v>250</v>
       </c>
       <c r="B51">
-        <v>28.05</v>
+        <v>28.548999999999999</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -13277,7 +13277,7 @@
         <v>255</v>
       </c>
       <c r="B52">
-        <v>28.454000000000001</v>
+        <v>28.968</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -13285,7 +13285,7 @@
         <v>260</v>
       </c>
       <c r="B53">
-        <v>28.850999999999999</v>
+        <v>29.381</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -13293,7 +13293,7 @@
         <v>265</v>
       </c>
       <c r="B54">
-        <v>29.244</v>
+        <v>29.789000000000001</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -13301,7 +13301,7 @@
         <v>270</v>
       </c>
       <c r="B55">
-        <v>29.634</v>
+        <v>30.196000000000002</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -13309,7 +13309,7 @@
         <v>275</v>
       </c>
       <c r="B56">
-        <v>30.024000000000001</v>
+        <v>30.602</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -13317,7 +13317,7 @@
         <v>280</v>
       </c>
       <c r="B57">
-        <v>30.414000000000001</v>
+        <v>31.010999999999999</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
@@ -13325,7 +13325,7 @@
         <v>285</v>
       </c>
       <c r="B58">
-        <v>30.806000000000001</v>
+        <v>31.422999999999998</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -13333,7 +13333,7 @@
         <v>290</v>
       </c>
       <c r="B59">
-        <v>31.202999999999999</v>
+        <v>31.841999999999999</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -13341,7 +13341,7 @@
         <v>295</v>
       </c>
       <c r="B60">
-        <v>31.609000000000002</v>
+        <v>32.271999999999998</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -13349,7 +13349,7 @@
         <v>300</v>
       </c>
       <c r="B61">
-        <v>32.027000000000001</v>
+        <v>32.718000000000004</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -13357,7 +13357,7 @@
         <v>305</v>
       </c>
       <c r="B62">
-        <v>32.465000000000003</v>
+        <v>33.188000000000002</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -13365,7 +13365,7 @@
         <v>310</v>
       </c>
       <c r="B63">
-        <v>32.933999999999997</v>
+        <v>33.695999999999998</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -13373,7 +13373,7 @@
         <v>315</v>
       </c>
       <c r="B64">
-        <v>33.451000000000001</v>
+        <v>34.262</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -13381,7 +13381,7 @@
         <v>320</v>
       </c>
       <c r="B65">
-        <v>34.048999999999999</v>
+        <v>34.926000000000002</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -13389,7 +13389,7 @@
         <v>325</v>
       </c>
       <c r="B66">
-        <v>34.786999999999999</v>
+        <v>35.762999999999998</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -13397,7 +13397,7 @@
         <v>330</v>
       </c>
       <c r="B67">
-        <v>35.783999999999999</v>
+        <v>36.914999999999999</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -13405,7 +13405,7 @@
         <v>335</v>
       </c>
       <c r="B68">
-        <v>37.253</v>
+        <v>38.594000000000001</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -13413,7 +13413,7 @@
         <v>340</v>
       </c>
       <c r="B69">
-        <v>39.216000000000001</v>
+        <v>40.335000000000001</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -13421,7 +13421,7 @@
         <v>345</v>
       </c>
       <c r="B70">
-        <v>39.292000000000002</v>
+        <v>39.052999999999997</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -13429,7 +13429,7 @@
         <v>350</v>
       </c>
       <c r="B71">
-        <v>36.472000000000001</v>
+        <v>36.476999999999997</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -13437,7 +13437,7 @@
         <v>355</v>
       </c>
       <c r="B72">
-        <v>35.003</v>
+        <v>35.529000000000003</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -13445,7 +13445,7 @@
         <v>360</v>
       </c>
       <c r="B73">
-        <v>34.695999999999998</v>
+        <v>35.433</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
@@ -13453,7 +13453,7 @@
         <v>365</v>
       </c>
       <c r="B74">
-        <v>34.798000000000002</v>
+        <v>35.622999999999998</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
@@ -13461,7 +13461,7 @@
         <v>370</v>
       </c>
       <c r="B75">
-        <v>35.034999999999997</v>
+        <v>35.911000000000001</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
@@ -13469,7 +13469,7 @@
         <v>375</v>
       </c>
       <c r="B76">
-        <v>35.32</v>
+        <v>36.232999999999997</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
@@ -13477,7 +13477,7 @@
         <v>380</v>
       </c>
       <c r="B77">
-        <v>35.622</v>
+        <v>36.567999999999998</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
@@ -13485,7 +13485,7 @@
         <v>385</v>
       </c>
       <c r="B78">
-        <v>35.930999999999997</v>
+        <v>36.908999999999999</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
@@ -13493,7 +13493,7 @@
         <v>390</v>
       </c>
       <c r="B79">
-        <v>36.243000000000002</v>
+        <v>37.253999999999998</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
@@ -13501,7 +13501,7 @@
         <v>395</v>
       </c>
       <c r="B80">
-        <v>36.558999999999997</v>
+        <v>37.603999999999999</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
@@ -13509,7 +13509,7 @@
         <v>400</v>
       </c>
       <c r="B81">
-        <v>36.880000000000003</v>
+        <v>37.960999999999999</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
@@ -13517,7 +13517,7 @@
         <v>405</v>
       </c>
       <c r="B82">
-        <v>37.207999999999998</v>
+        <v>38.328000000000003</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
@@ -13525,7 +13525,7 @@
         <v>410</v>
       </c>
       <c r="B83">
-        <v>37.546999999999997</v>
+        <v>38.707000000000001</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
@@ -13533,7 +13533,7 @@
         <v>415</v>
       </c>
       <c r="B84">
-        <v>37.9</v>
+        <v>39.100999999999999</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
@@ -13541,7 +13541,7 @@
         <v>420</v>
       </c>
       <c r="B85">
-        <v>38.270000000000003</v>
+        <v>39.511000000000003</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
@@ -13549,7 +13549,7 @@
         <v>425</v>
       </c>
       <c r="B86">
-        <v>38.656999999999996</v>
+        <v>39.930999999999997</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
@@ -13557,7 +13557,7 @@
         <v>430</v>
       </c>
       <c r="B87">
-        <v>39.058999999999997</v>
+        <v>40.334000000000003</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
@@ -13565,7 +13565,7 @@
         <v>435</v>
       </c>
       <c r="B88">
-        <v>39.447000000000003</v>
+        <v>40.642000000000003</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
@@ -13573,7 +13573,7 @@
         <v>440</v>
       </c>
       <c r="B89">
-        <v>39.737000000000002</v>
+        <v>40.683999999999997</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
@@ -13581,7 +13581,7 @@
         <v>445</v>
       </c>
       <c r="B90">
-        <v>39.74</v>
+        <v>40.335000000000001</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
@@ -13589,7 +13589,7 @@
         <v>450</v>
       </c>
       <c r="B91">
-        <v>39.322000000000003</v>
+        <v>39.939</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
@@ -13597,7 +13597,7 @@
         <v>455</v>
       </c>
       <c r="B92">
-        <v>38.866</v>
+        <v>39.963000000000001</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
@@ -13605,7 +13605,7 @@
         <v>460</v>
       </c>
       <c r="B93">
-        <v>38.844000000000001</v>
+        <v>40.362000000000002</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
@@ -13613,7 +13613,7 @@
         <v>465</v>
       </c>
       <c r="B94">
-        <v>39.186999999999998</v>
+        <v>40.929000000000002</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
@@ -13621,7 +13621,7 @@
         <v>470</v>
       </c>
       <c r="B95">
-        <v>39.69</v>
+        <v>41.557000000000002</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
@@ -13629,7 +13629,7 @@
         <v>475</v>
       </c>
       <c r="B96">
-        <v>40.253</v>
+        <v>42.210999999999999</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
@@ -13637,7 +13637,7 @@
         <v>480</v>
       </c>
       <c r="B97">
-        <v>40.843000000000004</v>
+        <v>42.872</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
@@ -13645,7 +13645,7 @@
         <v>485</v>
       </c>
       <c r="B98">
-        <v>41.445999999999998</v>
+        <v>43.503999999999998</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
@@ -13653,7 +13653,7 @@
         <v>490</v>
       </c>
       <c r="B99">
-        <v>42.039000000000001</v>
+        <v>44.03</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
@@ -13661,7 +13661,7 @@
         <v>495</v>
       </c>
       <c r="B100">
-        <v>42.563000000000002</v>
+        <v>44.351999999999997</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
@@ -13669,7 +13669,7 @@
         <v>500</v>
       </c>
       <c r="B101">
-        <v>42.927999999999997</v>
+        <v>44.472000000000001</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
@@ -13677,7 +13677,7 @@
         <v>505</v>
       </c>
       <c r="B102">
-        <v>43.085000000000001</v>
+        <v>44.567</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
@@ -13685,7 +13685,7 @@
         <v>510</v>
       </c>
       <c r="B103">
-        <v>43.155000000000001</v>
+        <v>44.746000000000002</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
@@ -13693,7 +13693,7 @@
         <v>515</v>
       </c>
       <c r="B104">
-        <v>43.311999999999998</v>
+        <v>44.786999999999999</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
@@ -13701,7 +13701,7 @@
         <v>520</v>
       </c>
       <c r="B105">
-        <v>43.488999999999997</v>
+        <v>44.383000000000003</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
@@ -13709,7 +13709,7 @@
         <v>525</v>
       </c>
       <c r="B106">
-        <v>43.343000000000004</v>
+        <v>43.695999999999998</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
@@ -13717,7 +13717,7 @@
         <v>530</v>
       </c>
       <c r="B107">
-        <v>42.73</v>
+        <v>43.16</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
@@ -13725,7 +13725,7 @@
         <v>535</v>
       </c>
       <c r="B108">
-        <v>42.027000000000001</v>
+        <v>42.927</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
@@ -13733,7 +13733,7 @@
         <v>540</v>
       </c>
       <c r="B109">
-        <v>41.58</v>
+        <v>42.935000000000002</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
@@ -13741,7 +13741,7 @@
         <v>545</v>
       </c>
       <c r="B110">
-        <v>41.418999999999997</v>
+        <v>43.106000000000002</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
@@ -13749,7 +13749,7 @@
         <v>550</v>
       </c>
       <c r="B111">
-        <v>41.454000000000001</v>
+        <v>43.406999999999996</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
@@ -13757,7 +13757,7 @@
         <v>555</v>
       </c>
       <c r="B112">
-        <v>41.622999999999998</v>
+        <v>43.826999999999998</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
@@ -13765,7 +13765,7 @@
         <v>560</v>
       </c>
       <c r="B113">
-        <v>41.904000000000003</v>
+        <v>44.35</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
@@ -13773,7 +13773,7 @@
         <v>565</v>
       </c>
       <c r="B114">
-        <v>42.289000000000001</v>
+        <v>44.96</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
@@ -13781,7 +13781,7 @@
         <v>570</v>
       </c>
       <c r="B115">
-        <v>42.765999999999998</v>
+        <v>45.636000000000003</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
@@ -13789,7 +13789,7 @@
         <v>575</v>
       </c>
       <c r="B116">
-        <v>43.322000000000003</v>
+        <v>46.337000000000003</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
@@ -13797,7 +13797,7 @@
         <v>580</v>
       </c>
       <c r="B117">
-        <v>43.947000000000003</v>
+        <v>46.924999999999997</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
@@ -13805,7 +13805,7 @@
         <v>585</v>
       </c>
       <c r="B118">
-        <v>44.618000000000002</v>
+        <v>47.125</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
@@ -13813,7 +13813,7 @@
         <v>590</v>
       </c>
       <c r="B119">
-        <v>45.234999999999999</v>
+        <v>46.988</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
@@ -13821,7 +13821,7 @@
         <v>595</v>
       </c>
       <c r="B120">
-        <v>45.546999999999997</v>
+        <v>47.021999999999998</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
@@ -13829,7 +13829,7 @@
         <v>600</v>
       </c>
       <c r="B121">
-        <v>45.457000000000001</v>
+        <v>47.396999999999998</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
@@ -13837,7 +13837,7 @@
         <v>605</v>
       </c>
       <c r="B122">
-        <v>45.404000000000003</v>
+        <v>48.07</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
@@ -13845,7 +13845,7 @@
         <v>610</v>
       </c>
       <c r="B123">
-        <v>45.686</v>
+        <v>49.066000000000003</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
@@ -13853,7 +13853,7 @@
         <v>615</v>
       </c>
       <c r="B124">
-        <v>46.314</v>
+        <v>50.180999999999997</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
@@ -13861,7 +13861,7 @@
         <v>620</v>
       </c>
       <c r="B125">
-        <v>47.307000000000002</v>
+        <v>50.231000000000002</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
@@ -13869,7 +13869,7 @@
         <v>625</v>
       </c>
       <c r="B126">
-        <v>48.533999999999999</v>
+        <v>48.692</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
@@ -13877,7 +13877,7 @@
         <v>630</v>
       </c>
       <c r="B127">
-        <v>48.920999999999999</v>
+        <v>47.145000000000003</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
@@ -13885,7 +13885,7 @@
         <v>635</v>
       </c>
       <c r="B128">
-        <v>47.533999999999999</v>
+        <v>46.368000000000002</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
@@ -13893,7 +13893,7 @@
         <v>640</v>
       </c>
       <c r="B129">
-        <v>45.776000000000003</v>
+        <v>46.222000000000001</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
@@ -13901,7 +13901,7 @@
         <v>645</v>
       </c>
       <c r="B130">
-        <v>44.674999999999997</v>
+        <v>46.433999999999997</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
@@ -13909,7 +13909,7 @@
         <v>650</v>
       </c>
       <c r="B131">
-        <v>44.223999999999997</v>
+        <v>46.81</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
@@ -13917,7 +13917,7 @@
         <v>655</v>
       </c>
       <c r="B132">
-        <v>44.201999999999998</v>
+        <v>47.225000000000001</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
@@ -13925,7 +13925,7 @@
         <v>660</v>
       </c>
       <c r="B133">
-        <v>44.420999999999999</v>
+        <v>47.6</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
@@ -13933,7 +13933,7 @@
         <v>665</v>
       </c>
       <c r="B134">
-        <v>44.753999999999998</v>
+        <v>47.886000000000003</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
@@ -13941,7 +13941,7 @@
         <v>670</v>
       </c>
       <c r="B135">
-        <v>45.119</v>
+        <v>48.061999999999998</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
@@ -13949,7 +13949,7 @@
         <v>675</v>
       </c>
       <c r="B136">
-        <v>45.456000000000003</v>
+        <v>48.143999999999998</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
@@ -13957,7 +13957,7 @@
         <v>680</v>
       </c>
       <c r="B137">
-        <v>45.726999999999997</v>
+        <v>48.173999999999999</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
@@ -13965,7 +13965,7 @@
         <v>685</v>
       </c>
       <c r="B138">
-        <v>45.91</v>
+        <v>48.209000000000003</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
@@ -13973,7 +13973,7 @@
         <v>690</v>
       </c>
       <c r="B139">
-        <v>46.003999999999998</v>
+        <v>48.295000000000002</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
@@ -13981,7 +13981,7 @@
         <v>695</v>
       </c>
       <c r="B140">
-        <v>46.034999999999997</v>
+        <v>48.454999999999998</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
@@ -13989,7 +13989,7 @@
         <v>700</v>
       </c>
       <c r="B141">
-        <v>46.045000000000002</v>
+        <v>48.695</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
@@ -13997,7 +13997,7 @@
         <v>705</v>
       </c>
       <c r="B142">
-        <v>46.073999999999998</v>
+        <v>49.005000000000003</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
@@ -14005,7 +14005,7 @@
         <v>710</v>
       </c>
       <c r="B143">
-        <v>46.152999999999999</v>
+        <v>49.366</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
@@ -14013,7 +14013,7 @@
         <v>715</v>
       </c>
       <c r="B144">
-        <v>46.298999999999999</v>
+        <v>49.753</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
@@ -14021,7 +14021,7 @@
         <v>720</v>
       </c>
       <c r="B145">
-        <v>46.512999999999998</v>
+        <v>50.124000000000002</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
@@ -14029,7 +14029,7 @@
         <v>725</v>
       </c>
       <c r="B146">
-        <v>46.790999999999997</v>
+        <v>50.405999999999999</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
@@ -14037,7 +14037,7 @@
         <v>730</v>
       </c>
       <c r="B147">
-        <v>47.122</v>
+        <v>50.506</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
@@ -14045,7 +14045,7 @@
         <v>735</v>
       </c>
       <c r="B148">
-        <v>47.487000000000002</v>
+        <v>50.417999999999999</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
@@ -14053,7 +14053,7 @@
         <v>740</v>
       </c>
       <c r="B149">
-        <v>47.845999999999997</v>
+        <v>50.273000000000003</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
@@ -14061,7 +14061,7 @@
         <v>745</v>
       </c>
       <c r="B150">
-        <v>48.118000000000002</v>
+        <v>50.21</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
@@ -14069,7 +14069,7 @@
         <v>750</v>
       </c>
       <c r="B151">
-        <v>48.2</v>
+        <v>50.271999999999998</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
@@ -14077,7 +14077,7 @@
         <v>755</v>
       </c>
       <c r="B152">
-        <v>48.072000000000003</v>
+        <v>50.436999999999998</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
@@ -14085,7 +14085,7 @@
         <v>760</v>
       </c>
       <c r="B153">
-        <v>47.86</v>
+        <v>50.673000000000002</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
@@ -14093,7 +14093,7 @@
         <v>765</v>
       </c>
       <c r="B154">
-        <v>47.707999999999998</v>
+        <v>50.951999999999998</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
@@ -14101,7 +14101,7 @@
         <v>770</v>
       </c>
       <c r="B155">
-        <v>47.664000000000001</v>
+        <v>51.253</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
@@ -14109,7 +14109,7 @@
         <v>775</v>
       </c>
       <c r="B156">
-        <v>47.716000000000001</v>
+        <v>51.563000000000002</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
@@ -14117,7 +14117,7 @@
         <v>780</v>
       </c>
       <c r="B157">
-        <v>47.838999999999999</v>
+        <v>51.871000000000002</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
@@ -14125,7 +14125,7 @@
         <v>785</v>
       </c>
       <c r="B158">
-        <v>48.01</v>
+        <v>52.173999999999999</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
@@ -14133,7 +14133,7 @@
         <v>790</v>
       </c>
       <c r="B159">
-        <v>48.212000000000003</v>
+        <v>52.472000000000001</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
@@ -14141,7 +14141,7 @@
         <v>795</v>
       </c>
       <c r="B160">
-        <v>48.435000000000002</v>
+        <v>52.768000000000001</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
@@ -14149,7 +14149,7 @@
         <v>800</v>
       </c>
       <c r="B161">
-        <v>48.67</v>
+        <v>53.067</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
@@ -14157,7 +14157,7 @@
         <v>805</v>
       </c>
       <c r="B162">
-        <v>48.911000000000001</v>
+        <v>53.36</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
@@ -14165,7 +14165,7 @@
         <v>810</v>
       </c>
       <c r="B163">
-        <v>49.155000000000001</v>
+        <v>53.624000000000002</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
@@ -14173,7 +14173,7 @@
         <v>815</v>
       </c>
       <c r="B164">
-        <v>49.404000000000003</v>
+        <v>53.804000000000002</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
@@ -14181,7 +14181,7 @@
         <v>820</v>
       </c>
       <c r="B165">
-        <v>49.661999999999999</v>
+        <v>53.844999999999999</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.25">
@@ -14189,7 +14189,7 @@
         <v>825</v>
       </c>
       <c r="B166">
-        <v>49.930999999999997</v>
+        <v>53.737000000000002</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
@@ -14197,7 +14197,7 @@
         <v>830</v>
       </c>
       <c r="B167">
-        <v>50.207000000000001</v>
+        <v>53.561999999999998</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
@@ -14205,7 +14205,7 @@
         <v>835</v>
       </c>
       <c r="B168">
-        <v>50.472000000000001</v>
+        <v>53.433999999999997</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
@@ -14213,7 +14213,7 @@
         <v>840</v>
       </c>
       <c r="B169">
-        <v>50.680999999999997</v>
+        <v>53.421999999999997</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
@@ -14221,7 +14221,7 @@
         <v>845</v>
       </c>
       <c r="B170">
-        <v>50.767000000000003</v>
+        <v>53.527999999999999</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
@@ -14229,7 +14229,7 @@
         <v>850</v>
       </c>
       <c r="B171">
-        <v>50.673999999999999</v>
+        <v>53.728999999999999</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
@@ -14237,7 +14237,7 @@
         <v>855</v>
       </c>
       <c r="B172">
-        <v>50.415999999999997</v>
+        <v>53.997</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
@@ -14245,7 +14245,7 @@
         <v>860</v>
       </c>
       <c r="B173">
-        <v>50.097000000000001</v>
+        <v>54.308999999999997</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
@@ -14253,7 +14253,7 @@
         <v>865</v>
       </c>
       <c r="B174">
-        <v>49.83</v>
+        <v>54.625</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
@@ -14261,7 +14261,7 @@
         <v>870</v>
       </c>
       <c r="B175">
-        <v>49.670999999999999</v>
+        <v>54.87</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
@@ -14269,7 +14269,7 @@
         <v>875</v>
       </c>
       <c r="B176">
-        <v>49.622</v>
+        <v>54.954999999999998</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
@@ -14277,7 +14277,7 @@
         <v>880</v>
       </c>
       <c r="B177">
-        <v>49.661999999999999</v>
+        <v>54.911000000000001</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
@@ -14285,7 +14285,7 @@
         <v>885</v>
       </c>
       <c r="B178">
-        <v>49.765999999999998</v>
+        <v>54.881999999999998</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
@@ -14293,7 +14293,7 @@
         <v>890</v>
       </c>
       <c r="B179">
-        <v>49.912999999999997</v>
+        <v>54.96</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
@@ -14301,7 +14301,7 @@
         <v>895</v>
       </c>
       <c r="B180">
-        <v>50.08</v>
+        <v>55.119</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
@@ -14309,7 +14309,7 @@
         <v>900</v>
       </c>
       <c r="B181">
-        <v>50.228999999999999</v>
+        <v>55.335999999999999</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
@@ -14317,7 +14317,7 @@
         <v>905</v>
       </c>
       <c r="B182">
-        <v>50.295999999999999</v>
+        <v>55.698</v>
       </c>
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
@@ -14325,7 +14325,7 @@
         <v>910</v>
       </c>
       <c r="B183">
-        <v>50.246000000000002</v>
+        <v>56.161000000000001</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
@@ -14333,7 +14333,7 @@
         <v>915</v>
       </c>
       <c r="B184">
-        <v>50.146000000000001</v>
+        <v>56.621000000000002</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
@@ -14341,7 +14341,7 @@
         <v>920</v>
       </c>
       <c r="B185">
-        <v>50.113999999999997</v>
+        <v>57.014000000000003</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
@@ -14349,7 +14349,7 @@
         <v>925</v>
       </c>
       <c r="B186">
-        <v>50.201999999999998</v>
+        <v>57.35</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
@@ -14357,7 +14357,7 @@
         <v>930</v>
       </c>
       <c r="B187">
-        <v>50.343000000000004</v>
+        <v>57.68</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
@@ -14365,7 +14365,7 @@
         <v>935</v>
       </c>
       <c r="B188">
-        <v>50.468000000000004</v>
+        <v>58.037999999999997</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
@@ -14373,7 +14373,7 @@
         <v>940</v>
       </c>
       <c r="B189">
-        <v>50.661999999999999</v>
+        <v>58.433999999999997</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
@@ -14381,7 +14381,7 @@
         <v>945</v>
       </c>
       <c r="B190">
-        <v>50.957000000000001</v>
+        <v>58.862000000000002</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
@@ -14389,7 +14389,7 @@
         <v>950</v>
       </c>
       <c r="B191">
-        <v>51.283000000000001</v>
+        <v>59.305999999999997</v>
       </c>
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
@@ -14397,7 +14397,7 @@
         <v>955</v>
       </c>
       <c r="B192">
-        <v>51.564999999999998</v>
+        <v>59.750999999999998</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
@@ -14405,7 +14405,7 @@
         <v>960</v>
       </c>
       <c r="B193">
-        <v>51.78</v>
+        <v>60.183999999999997</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
@@ -14413,7 +14413,7 @@
         <v>965</v>
       </c>
       <c r="B194">
-        <v>51.959000000000003</v>
+        <v>60.593000000000004</v>
       </c>
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
@@ -14421,7 +14421,7 @@
         <v>970</v>
       </c>
       <c r="B195">
-        <v>52.134999999999998</v>
+        <v>60.970999999999997</v>
       </c>
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
@@ -14429,7 +14429,7 @@
         <v>975</v>
       </c>
       <c r="B196">
-        <v>52.329000000000001</v>
+        <v>61.32</v>
       </c>
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
@@ -14437,7 +14437,7 @@
         <v>980</v>
       </c>
       <c r="B197">
-        <v>52.561</v>
+        <v>61.655999999999999</v>
       </c>
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
@@ -14445,7 +14445,7 @@
         <v>985</v>
       </c>
       <c r="B198">
-        <v>52.826999999999998</v>
+        <v>62.005000000000003</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
@@ -14453,7 +14453,7 @@
         <v>990</v>
       </c>
       <c r="B199">
-        <v>53.110999999999997</v>
+        <v>62.399000000000001</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
@@ -14461,7 +14461,7 @@
         <v>995</v>
       </c>
       <c r="B200">
-        <v>53.408000000000001</v>
+        <v>62.853999999999999</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
@@ -14469,7 +14469,7 @@
         <v>1000</v>
       </c>
       <c r="B201">
-        <v>53.712000000000003</v>
+        <v>63.354999999999997</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.25">
@@ -14477,7 +14477,7 @@
         <v>1005</v>
       </c>
       <c r="B202">
-        <v>54.02</v>
+        <v>63.831000000000003</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
@@ -14485,7 +14485,7 @@
         <v>1010</v>
       </c>
       <c r="B203">
-        <v>54.328000000000003</v>
+        <v>64.176000000000002</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
@@ -14493,7 +14493,7 @@
         <v>1015</v>
       </c>
       <c r="B204">
-        <v>54.634</v>
+        <v>64.331000000000003</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
@@ -14501,7 +14501,7 @@
         <v>1020</v>
       </c>
       <c r="B205">
-        <v>54.936999999999998</v>
+        <v>64.337999999999994</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.25">
@@ -14509,7 +14509,7 @@
         <v>1025</v>
       </c>
       <c r="B206">
-        <v>55.243000000000002</v>
+        <v>64.283000000000001</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
@@ -14517,7 +14517,7 @@
         <v>1030</v>
       </c>
       <c r="B207">
-        <v>55.563000000000002</v>
+        <v>64.218000000000004</v>
       </c>
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
@@ -14525,7 +14525,7 @@
         <v>1035</v>
       </c>
       <c r="B208">
-        <v>55.915999999999997</v>
+        <v>64.150999999999996</v>
       </c>
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
@@ -14533,7 +14533,7 @@
         <v>1040</v>
       </c>
       <c r="B209">
-        <v>56.323999999999998</v>
+        <v>64.061000000000007</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
@@ -14541,7 +14541,7 @@
         <v>1045</v>
       </c>
       <c r="B210">
-        <v>56.804000000000002</v>
+        <v>63.902000000000001</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
@@ -14549,7 +14549,7 @@
         <v>1050</v>
       </c>
       <c r="B211">
-        <v>57.356999999999999</v>
+        <v>63.622999999999998</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
@@ -14557,7 +14557,7 @@
         <v>1055</v>
       </c>
       <c r="B212">
-        <v>57.957000000000001</v>
+        <v>63.209000000000003</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
@@ -14565,7 +14565,7 @@
         <v>1060</v>
       </c>
       <c r="B213">
-        <v>58.55</v>
+        <v>62.744999999999997</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.25">
@@ -14573,7 +14573,7 @@
         <v>1065</v>
       </c>
       <c r="B214">
-        <v>59.09</v>
+        <v>62.37</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
@@ -14581,7 +14581,7 @@
         <v>1070</v>
       </c>
       <c r="B215">
-        <v>59.564999999999998</v>
+        <v>62.104999999999997</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
@@ -14589,7 +14589,7 @@
         <v>1075</v>
       </c>
       <c r="B216">
-        <v>59.997999999999998</v>
+        <v>61.853999999999999</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
@@ -14597,7 +14597,7 @@
         <v>1080</v>
       </c>
       <c r="B217">
-        <v>60.414999999999999</v>
+        <v>61.597999999999999</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.25">
@@ -14605,7 +14605,7 @@
         <v>1085</v>
       </c>
       <c r="B218">
-        <v>60.838999999999999</v>
+        <v>61.372999999999998</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
@@ -14613,7 +14613,7 @@
         <v>1090</v>
       </c>
       <c r="B219">
-        <v>61.277000000000001</v>
+        <v>61.197000000000003</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
@@ -14621,7 +14621,7 @@
         <v>1095</v>
       </c>
       <c r="B220">
-        <v>61.71</v>
+        <v>61.069000000000003</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
@@ -14629,7 +14629,7 @@
         <v>1100</v>
       </c>
       <c r="B221">
-        <v>62.088000000000001</v>
+        <v>60.988</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
@@ -14637,7 +14637,7 @@
         <v>1105</v>
       </c>
       <c r="B222">
-        <v>62.326000000000001</v>
+        <v>60.953000000000003</v>
       </c>
     </row>
     <row r="223" spans="1:2" x14ac:dyDescent="0.25">
@@ -14645,7 +14645,7 @@
         <v>1110</v>
       </c>
       <c r="B223">
-        <v>62.345999999999997</v>
+        <v>60.951999999999998</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.25">
@@ -14653,7 +14653,7 @@
         <v>1115</v>
       </c>
       <c r="B224">
-        <v>62.155999999999999</v>
+        <v>60.956000000000003</v>
       </c>
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
@@ -14661,7 +14661,7 @@
         <v>1120</v>
       </c>
       <c r="B225">
-        <v>61.893999999999998</v>
+        <v>60.927</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
@@ -14669,7 +14669,7 @@
         <v>1125</v>
       </c>
       <c r="B226">
-        <v>61.707000000000001</v>
+        <v>60.847000000000001</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.25">
@@ -14677,7 +14677,7 @@
         <v>1130</v>
       </c>
       <c r="B227">
-        <v>61.58</v>
+        <v>60.726999999999997</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
@@ -14685,7 +14685,7 @@
         <v>1135</v>
       </c>
       <c r="B228">
-        <v>61.375999999999998</v>
+        <v>60.601999999999997</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
@@ -14693,7 +14693,7 @@
         <v>1140</v>
       </c>
       <c r="B229">
-        <v>61.051000000000002</v>
+        <v>60.503999999999998</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
@@ -14701,7 +14701,7 @@
         <v>1145</v>
       </c>
       <c r="B230">
-        <v>60.722000000000001</v>
+        <v>60.441000000000003</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.25">
@@ -14709,7 +14709,7 @@
         <v>1150</v>
       </c>
       <c r="B231">
-        <v>60.466000000000001</v>
+        <v>60.405000000000001</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
@@ -14717,7 +14717,7 @@
         <v>1155</v>
       </c>
       <c r="B232">
-        <v>60.28</v>
+        <v>60.362000000000002</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.25">
@@ -14725,7 +14725,7 @@
         <v>1160</v>
       </c>
       <c r="B233">
-        <v>60.140999999999998</v>
+        <v>60.234999999999999</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
@@ -14733,7 +14733,7 @@
         <v>1165</v>
       </c>
       <c r="B234">
-        <v>60.04</v>
+        <v>59.924999999999997</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.25">
@@ -14741,7 +14741,7 @@
         <v>1170</v>
       </c>
       <c r="B235">
-        <v>59.976999999999997</v>
+        <v>59.473999999999997</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.25">
@@ -14749,7 +14749,7 @@
         <v>1175</v>
       </c>
       <c r="B236">
-        <v>59.953000000000003</v>
+        <v>59.058</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.25">
@@ -14757,7 +14757,7 @@
         <v>1180</v>
       </c>
       <c r="B237">
-        <v>59.948999999999998</v>
+        <v>58.77</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.25">
@@ -14765,7 +14765,7 @@
         <v>1185</v>
       </c>
       <c r="B238">
-        <v>59.923000000000002</v>
+        <v>58.601999999999997</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.25">
@@ -14773,7 +14773,7 @@
         <v>1190</v>
       </c>
       <c r="B239">
-        <v>59.828000000000003</v>
+        <v>58.523000000000003</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.25">
@@ -14781,7 +14781,7 @@
         <v>1195</v>
       </c>
       <c r="B240">
-        <v>59.646999999999998</v>
+        <v>58.512</v>
       </c>
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.25">
@@ -14789,7 +14789,7 @@
         <v>1200</v>
       </c>
       <c r="B241">
-        <v>59.405999999999999</v>
+        <v>58.56</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.25">
@@ -14797,7 +14797,7 @@
         <v>1205</v>
       </c>
       <c r="B242">
-        <v>59.152999999999999</v>
+        <v>58.671999999999997</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.25">
@@ -14805,7 +14805,7 @@
         <v>1210</v>
       </c>
       <c r="B243">
-        <v>58.927999999999997</v>
+        <v>58.847999999999999</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.25">
@@ -14813,7 +14813,7 @@
         <v>1215</v>
       </c>
       <c r="B244">
-        <v>58.746000000000002</v>
+        <v>59.036999999999999</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.25">
@@ -14821,7 +14821,7 @@
         <v>1220</v>
       </c>
       <c r="B245">
-        <v>58.587000000000003</v>
+        <v>59.142000000000003</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.25">
@@ -14829,7 +14829,7 @@
         <v>1225</v>
       </c>
       <c r="B246">
-        <v>58.393999999999998</v>
+        <v>59.112000000000002</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.25">
@@ -14837,7 +14837,7 @@
         <v>1230</v>
       </c>
       <c r="B247">
-        <v>58.07</v>
+        <v>58.970999999999997</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.25">
@@ -14845,7 +14845,7 @@
         <v>1235</v>
       </c>
       <c r="B248">
-        <v>57.542000000000002</v>
+        <v>58.77</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.25">
@@ -14853,7 +14853,7 @@
         <v>1240</v>
       </c>
       <c r="B249">
-        <v>56.898000000000003</v>
+        <v>58.554000000000002</v>
       </c>
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.25">
@@ -14861,7 +14861,7 @@
         <v>1245</v>
       </c>
       <c r="B250">
-        <v>56.317999999999998</v>
+        <v>58.350999999999999</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.25">
@@ -14869,7 +14869,7 @@
         <v>1250</v>
       </c>
       <c r="B251">
-        <v>55.881</v>
+        <v>58.173999999999999</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.25">
@@ -14877,7 +14877,7 @@
         <v>1255</v>
       </c>
       <c r="B252">
-        <v>55.567</v>
+        <v>58.023000000000003</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.25">
@@ -14885,7 +14885,7 @@
         <v>1260</v>
       </c>
       <c r="B253">
-        <v>55.337000000000003</v>
+        <v>57.884</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.25">
@@ -14893,7 +14893,7 @@
         <v>1265</v>
       </c>
       <c r="B254">
-        <v>55.168999999999997</v>
+        <v>57.731000000000002</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.25">
@@ -14901,7 +14901,7 @@
         <v>1270</v>
       </c>
       <c r="B255">
-        <v>55.052</v>
+        <v>57.536999999999999</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.25">
@@ -14909,7 +14909,7 @@
         <v>1275</v>
       </c>
       <c r="B256">
-        <v>54.98</v>
+        <v>57.296999999999997</v>
       </c>
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.25">
@@ -14917,7 +14917,7 @@
         <v>1280</v>
       </c>
       <c r="B257">
-        <v>54.948</v>
+        <v>57.070999999999998</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
@@ -14925,7 +14925,7 @@
         <v>1285</v>
       </c>
       <c r="B258">
-        <v>54.957000000000001</v>
+        <v>56.901000000000003</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
@@ -14933,7 +14933,7 @@
         <v>1290</v>
       </c>
       <c r="B259">
-        <v>55.012999999999998</v>
+        <v>56.713999999999999</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
@@ -14941,7 +14941,7 @@
         <v>1295</v>
       </c>
       <c r="B260">
-        <v>55.125999999999998</v>
+        <v>56.497999999999998</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
@@ -14949,7 +14949,7 @@
         <v>1300</v>
       </c>
       <c r="B261">
-        <v>55.280999999999999</v>
+        <v>56.301000000000002</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.25">
@@ -14957,7 +14957,7 @@
         <v>1305</v>
       </c>
       <c r="B262">
-        <v>55.427999999999997</v>
+        <v>56.168999999999997</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.25">
@@ -14965,7 +14965,7 @@
         <v>1310</v>
       </c>
       <c r="B263">
-        <v>55.506999999999998</v>
+        <v>56.113</v>
       </c>
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
@@ -14973,7 +14973,7 @@
         <v>1315</v>
       </c>
       <c r="B264">
-        <v>55.494</v>
+        <v>56.097999999999999</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
@@ -14981,7 +14981,7 @@
         <v>1320</v>
       </c>
       <c r="B265">
-        <v>55.4</v>
+        <v>56.072000000000003</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
@@ -14989,7 +14989,7 @@
         <v>1325</v>
       </c>
       <c r="B266">
-        <v>55.252000000000002</v>
+        <v>56.005000000000003</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
@@ -14997,7 +14997,7 @@
         <v>1330</v>
       </c>
       <c r="B267">
-        <v>55.08</v>
+        <v>55.893000000000001</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
@@ -15005,7 +15005,7 @@
         <v>1335</v>
       </c>
       <c r="B268">
-        <v>54.902999999999999</v>
+        <v>55.738</v>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.25">
@@ -15013,7 +15013,7 @@
         <v>1340</v>
       </c>
       <c r="B269">
-        <v>54.738</v>
+        <v>55.546999999999997</v>
       </c>
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.25">
@@ -15021,7 +15021,7 @@
         <v>1345</v>
       </c>
       <c r="B270">
-        <v>54.591000000000001</v>
+        <v>55.325000000000003</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.25">
@@ -15029,7 +15029,7 @@
         <v>1350</v>
       </c>
       <c r="B271">
-        <v>54.462000000000003</v>
+        <v>55.085999999999999</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.25">
@@ -15037,7 +15037,7 @@
         <v>1355</v>
       </c>
       <c r="B272">
-        <v>54.344999999999999</v>
+        <v>54.844000000000001</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.25">
@@ -15045,7 +15045,7 @@
         <v>1360</v>
       </c>
       <c r="B273">
-        <v>54.228000000000002</v>
+        <v>54.616999999999997</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.25">
@@ -15053,7 +15053,7 @@
         <v>1365</v>
       </c>
       <c r="B274">
-        <v>54.091999999999999</v>
+        <v>54.415999999999997</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.25">
@@ -15061,7 +15061,7 @@
         <v>1370</v>
       </c>
       <c r="B275">
-        <v>53.915999999999997</v>
+        <v>54.247999999999998</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.25">
@@ -15069,7 +15069,7 @@
         <v>1375</v>
       </c>
       <c r="B276">
-        <v>53.697000000000003</v>
+        <v>54.113</v>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.25">
@@ -15077,7 +15077,7 @@
         <v>1380</v>
       </c>
       <c r="B277">
-        <v>53.470999999999997</v>
+        <v>54.008000000000003</v>
       </c>
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.25">
@@ -15085,7 +15085,7 @@
         <v>1385</v>
       </c>
       <c r="B278">
-        <v>53.31</v>
+        <v>53.923000000000002</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.25">
@@ -15093,7 +15093,7 @@
         <v>1390</v>
       </c>
       <c r="B279">
-        <v>53.24</v>
+        <v>53.847999999999999</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.25">
@@ -15101,7 +15101,7 @@
         <v>1395</v>
       </c>
       <c r="B280">
-        <v>53.206000000000003</v>
+        <v>53.774000000000001</v>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.25">
@@ -15109,7 +15109,7 @@
         <v>1400</v>
       </c>
       <c r="B281">
-        <v>53.168999999999997</v>
+        <v>53.691000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>